<commit_message>
modified:   data/chapter2/FRED/subsets/final.xlsx 	modified:   notebooks/chapter_02/taxonomiccoverage.ipynb 	renamed:    notebooks/chapter_02/paper-draft.ipynb -> notebooks/chapter_02/wrangling.ipynb
</commit_message>
<xml_diff>
--- a/data/chapter2/FRED/subsets/final.xlsx
+++ b/data/chapter2/FRED/subsets/final.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://westernsydneyedu-my.sharepoint.com/personal/90963425_westernsydney_edu_au/Documents/PhD/code/data/chapter2/FRED/subsets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="44" documentId="11_08F17C2912DD3A461500DFF0505ED87656C112D0" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FD2D81CB-D107-4DB8-B989-75024AA83688}"/>
+  <xr:revisionPtr revIDLastSave="48" documentId="11_08F17C2912DD3A461500DFF0505ED87656C112D0" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F8D966E6-8F09-4977-9AF3-043B6DDE38D6}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -8850,6 +8850,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -25081,10 +25085,10 @@
         <v>0.11843955338983669</v>
       </c>
       <c r="J501" t="s">
-        <v>15</v>
+        <v>33</v>
       </c>
       <c r="K501" t="s">
-        <v>24</v>
+        <v>34</v>
       </c>
     </row>
     <row r="502" spans="1:12" x14ac:dyDescent="0.25">

</xml_diff>